<commit_message>
DDFW & DataProvider PRGS
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestDataNew.xlsx
+++ b/src/test/resources/testdata/TestDataNew.xlsx
@@ -3,22 +3,23 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nalla\git\HybridFW_670Batch\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{033734E7-DC52-4C31-B96E-96171EE8899E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87C5129E-F0C9-45ED-98CB-1A862E2EF943}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7800" yWindow="1005" windowWidth="15375" windowHeight="7785" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Testabc" sheetId="2" r:id="rId2"/>
+    <sheet name="new" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t>Test(row,column)</t>
   </si>
@@ -68,12 +69,34 @@
   </si>
   <si>
     <t>ew634yhgcgSreeni@gmail.com</t>
+  </si>
+  <si>
+    <t>Results</t>
+  </si>
+  <si>
+    <t>sabhitha04@gmail.com</t>
+  </si>
+  <si>
+    <t>jansi3006</t>
+  </si>
+  <si>
+    <t>ytest1@gmail.com</t>
+  </si>
+  <si>
+    <t>ytest1@</t>
+  </si>
+  <si>
+    <t>Fail / Invalid credentils</t>
+  </si>
+  <si>
+    <t>Pass / Valid credentils</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -421,51 +444,51 @@
   <dimension ref="A1:J13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="3.0"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="17.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="10.5703125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="12.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1">
+      <c r="A1" s="0">
         <v>0</v>
       </c>
-      <c r="B1">
+      <c r="B1" s="0">
         <v>1</v>
       </c>
-      <c r="C1">
+      <c r="C1" s="0">
         <v>2</v>
       </c>
-      <c r="D1">
+      <c r="D1" s="0">
         <v>3</v>
       </c>
-      <c r="E1">
+      <c r="E1" s="0">
         <v>4</v>
       </c>
-      <c r="F1">
+      <c r="F1" s="0">
         <v>5</v>
       </c>
-      <c r="G1">
+      <c r="G1" s="0">
         <v>6</v>
       </c>
-      <c r="H1">
+      <c r="H1" s="0">
         <v>7</v>
       </c>
-      <c r="I1">
+      <c r="I1" s="0">
         <v>8</v>
       </c>
-      <c r="J1">
+      <c r="J1" s="0">
         <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2">
+      <c r="A2" s="0">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3">
+      <c r="A3" s="0">
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
@@ -473,7 +496,7 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4">
+      <c r="A4" s="0">
         <v>3</v>
       </c>
       <c r="D4" s="1" t="s">
@@ -481,53 +504,53 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5">
+      <c r="A5" s="0">
         <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6">
+      <c r="A6" s="0">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7">
+      <c r="A7" s="0">
         <v>6</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" t="s" s="0">
         <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8">
+      <c r="A8" s="0">
         <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9">
+      <c r="A9" s="0">
         <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10">
+      <c r="A10" s="0">
         <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11">
+      <c r="A11" s="0">
         <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12">
+      <c r="A12" s="0">
         <v>11</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" t="s" s="0">
         <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13">
+      <c r="A13" s="0">
         <v>12</v>
       </c>
     </row>
@@ -538,52 +561,89 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6CE8E28-DCBE-4E5A-B9BC-25002C6FCFE9}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="34.140625" customWidth="1"/>
-    <col min="3" max="3" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" customWidth="true" width="34.140625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="21.5703125"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="14.7109375"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C1" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C2" t="s" s="0">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C3" t="s" s="0">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" t="s" s="0">
         <v>9</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C4" t="s" s="0">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" t="s" s="0">
         <v>10</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -593,8 +653,20 @@
     <hyperlink ref="A3" r:id="rId2" xr:uid="{8F175B4D-76A5-4C1B-8C7B-C56CE514603C}"/>
     <hyperlink ref="A4" r:id="rId3" xr:uid="{45129A2F-FFEC-4858-B56A-D647DC8B56A4}"/>
     <hyperlink ref="A5" r:id="rId4" xr:uid="{C7EB4EFE-2D07-4586-85A4-8D0751893BFB}"/>
+    <hyperlink ref="A6" r:id="rId5" xr:uid="{6D11B028-47A0-43A4-A0D6-1FDB95F4EDE3}"/>
+    <hyperlink ref="A7" r:id="rId6" xr:uid="{4B0F9CE2-ED4E-4F4A-9ABB-29A0C66DF651}"/>
+    <hyperlink ref="B7" r:id="rId7" xr:uid="{8B92CE79-258C-41A6-9BD8-048EC5AF1506}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId5"/>
+  <pageSetup orientation="portrait" r:id="rId8"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCF2B367-2BA1-44B8-BD3A-EAD3E2901868}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>